<commit_message>
Add workshop app (API, web, demos)
Introduce a local "workshop" application: a FastAPI standalone backend with analyzer-compare and pipeline routers/services, a React (CRA + Fluent UI) web frontend, and supporting helpers. Adds .env examples, VSCode settings, README with setup/run instructions, demo SOV preprocessing notebooks/scripts and reference outputs, feedback/underwriting artifacts, package.json/package-lock for the web, and requirements.txt. Enables local comparison of Azure Document Intelligence and Content Understanding analyzers and includes pipeline examples and utilities for running and inspecting results.
</commit_message>
<xml_diff>
--- a/demo/sov/attachments/01_acme_SOV.xlsx
+++ b/demo/sov/attachments/01_acme_SOV.xlsx
@@ -211,6 +211,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -660,10 +663,8 @@
           <t>Number of Locations</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>22 (+3 see embedded image below)</t>
-        </is>
+      <c r="B13" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="14">

</xml_diff>